<commit_message>
Align metadata and workbooks with current ALE contract
</commit_message>
<xml_diff>
--- a/artifacts/任务规格转化.xlsx
+++ b/artifacts/任务规格转化.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="R35784765ce8247da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="R6670911766ae4387"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -443,7 +443,7 @@
     </x:row>
     <x:row r="18" ht="33" customHeight="1">
       <x:c r="A18" s="4" t="str">
-        <x:v>结果核对</x:v>
+        <x:v>可验证点</x:v>
       </x:c>
       <x:c r="B18" s="4" t="str">
         <x:v>对象年龄、决策原因、批次成员、路径、容量和manifest均可从输入与业务明细复算</x:v>
@@ -451,7 +451,7 @@
     </x:row>
     <x:row r="19" ht="33" customHeight="1">
       <x:c r="A19" s="4" t="str">
-        <x:v>实现自由度</x:v>
+        <x:v>不适合作为评分点的内容</x:v>
       </x:c>
       <x:c r="B19" s="4" t="str">
         <x:v>函数拆分、内部容器、对象键序、CSV字段引用符和本机路径可以不同</x:v>

</xml_diff>